<commit_message>
atualiza volumes loa com ppo - 25092026.3
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/bancos/SISOR/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -884,10 +884,10 @@
         </is>
       </c>
       <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
         <v>60000</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -952,10 +952,10 @@
         </is>
       </c>
       <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
         <v>197857</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1020,10 +1020,10 @@
         </is>
       </c>
       <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
         <v>1929103</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1088,10 +1088,10 @@
         </is>
       </c>
       <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
         <v>1929103</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1156,10 +1156,10 @@
         </is>
       </c>
       <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
         <v>41022</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1224,10 +1224,10 @@
         </is>
       </c>
       <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
         <v>100000</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -4824,10 +4824,10 @@
         </is>
       </c>
       <c r="Q72" t="n">
-        <v>280106</v>
+        <v>0</v>
       </c>
       <c r="R72" t="n">
-        <v>519640</v>
+        <v>799746</v>
       </c>
     </row>
     <row r="73">
@@ -4884,10 +4884,10 @@
         </is>
       </c>
       <c r="Q73" t="n">
-        <v>894720</v>
+        <v>0</v>
       </c>
       <c r="R73" t="n">
-        <v>4087644</v>
+        <v>4982364</v>
       </c>
     </row>
     <row r="74">
@@ -4944,10 +4944,10 @@
         </is>
       </c>
       <c r="Q74" t="n">
-        <v>8264640</v>
+        <v>0</v>
       </c>
       <c r="R74" t="n">
-        <v>19153735</v>
+        <v>27418375</v>
       </c>
     </row>
     <row r="75">
@@ -5004,10 +5004,10 @@
         </is>
       </c>
       <c r="Q75" t="n">
-        <v>3155040</v>
+        <v>0</v>
       </c>
       <c r="R75" t="n">
-        <v>23943007</v>
+        <v>27098047</v>
       </c>
     </row>
     <row r="76">
@@ -5064,10 +5064,10 @@
         </is>
       </c>
       <c r="Q76" t="n">
-        <v>4840800</v>
+        <v>0</v>
       </c>
       <c r="R76" t="n">
-        <v>26593690</v>
+        <v>31434490</v>
       </c>
     </row>
     <row r="77">
@@ -5124,10 +5124,10 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>613500</v>
+        <v>0</v>
       </c>
       <c r="R77" t="n">
-        <v>2870210</v>
+        <v>3483710</v>
       </c>
     </row>
     <row r="78">
@@ -5184,10 +5184,10 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>5963400</v>
+        <v>0</v>
       </c>
       <c r="R78" t="n">
-        <v>23280000</v>
+        <v>29243400</v>
       </c>
     </row>
     <row r="79">
@@ -5244,10 +5244,10 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>3620820</v>
+        <v>0</v>
       </c>
       <c r="R79" t="n">
-        <v>19100000</v>
+        <v>22720820</v>
       </c>
     </row>
     <row r="80">
@@ -5361,10 +5361,10 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>1839798</v>
+        <v>0</v>
       </c>
       <c r="R81" t="n">
-        <v>3269655</v>
+        <v>5109453</v>
       </c>
     </row>
     <row r="82">
@@ -5421,10 +5421,10 @@
         </is>
       </c>
       <c r="Q82" t="n">
+        <v>0</v>
+      </c>
+      <c r="R82" t="n">
         <v>222899</v>
-      </c>
-      <c r="R82" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -6429,10 +6429,10 @@
         </is>
       </c>
       <c r="Q99" t="n">
+        <v>0</v>
+      </c>
+      <c r="R99" t="n">
         <v>299895</v>
-      </c>
-      <c r="R99" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -6489,10 +6489,10 @@
         </is>
       </c>
       <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="n">
         <v>4565604</v>
-      </c>
-      <c r="R100" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -6549,10 +6549,10 @@
         </is>
       </c>
       <c r="Q101" t="n">
-        <v>6286532</v>
+        <v>0</v>
       </c>
       <c r="R101" t="n">
-        <v>2728583</v>
+        <v>9015115</v>
       </c>
     </row>
     <row r="102">
@@ -6609,10 +6609,10 @@
         </is>
       </c>
       <c r="Q102" t="n">
+        <v>0</v>
+      </c>
+      <c r="R102" t="n">
         <v>193263</v>
-      </c>
-      <c r="R102" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -6780,10 +6780,10 @@
         </is>
       </c>
       <c r="Q105" t="n">
-        <v>904245</v>
+        <v>0</v>
       </c>
       <c r="R105" t="n">
-        <v>44308050</v>
+        <v>45212295</v>
       </c>
     </row>
     <row r="106">
@@ -6837,10 +6837,10 @@
         </is>
       </c>
       <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="n">
         <v>6999284</v>
-      </c>
-      <c r="R106" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -6894,10 +6894,10 @@
         </is>
       </c>
       <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="n">
         <v>651694</v>
-      </c>
-      <c r="R107" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -6951,10 +6951,10 @@
         </is>
       </c>
       <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
         <v>651694</v>
-      </c>
-      <c r="R108" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -7008,10 +7008,10 @@
         </is>
       </c>
       <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
         <v>1472757</v>
-      </c>
-      <c r="R109" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -7065,10 +7065,10 @@
         </is>
       </c>
       <c r="Q110" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" t="n">
         <v>651694</v>
-      </c>
-      <c r="R110" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -7122,10 +7122,10 @@
         </is>
       </c>
       <c r="Q111" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" t="n">
         <v>18572878</v>
-      </c>
-      <c r="R111" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -7643,10 +7643,10 @@
         </is>
       </c>
       <c r="Q120" t="n">
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="R120" t="n">
-        <v>19850000</v>
+        <v>20000000</v>
       </c>
     </row>
     <row r="121">
@@ -7945,10 +7945,10 @@
         </is>
       </c>
       <c r="Q125" t="n">
+        <v>0</v>
+      </c>
+      <c r="R125" t="n">
         <v>350000</v>
-      </c>
-      <c r="R125" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="126">
@@ -8010,10 +8010,10 @@
         </is>
       </c>
       <c r="Q126" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R126" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="127">
@@ -8700,10 +8700,10 @@
         </is>
       </c>
       <c r="Q138" t="n">
+        <v>0</v>
+      </c>
+      <c r="R138" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R138" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -8757,10 +8757,10 @@
         </is>
       </c>
       <c r="Q139" t="n">
+        <v>0</v>
+      </c>
+      <c r="R139" t="n">
         <v>143000</v>
-      </c>
-      <c r="R139" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -8814,10 +8814,10 @@
         </is>
       </c>
       <c r="Q140" t="n">
+        <v>0</v>
+      </c>
+      <c r="R140" t="n">
         <v>5876140</v>
-      </c>
-      <c r="R140" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="141">
@@ -8871,10 +8871,10 @@
         </is>
       </c>
       <c r="Q141" t="n">
+        <v>0</v>
+      </c>
+      <c r="R141" t="n">
         <v>1132500</v>
-      </c>
-      <c r="R141" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -8928,10 +8928,10 @@
         </is>
       </c>
       <c r="Q142" t="n">
+        <v>0</v>
+      </c>
+      <c r="R142" t="n">
         <v>34710000</v>
-      </c>
-      <c r="R142" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -8985,10 +8985,10 @@
         </is>
       </c>
       <c r="Q143" t="n">
+        <v>0</v>
+      </c>
+      <c r="R143" t="n">
         <v>59000000</v>
-      </c>
-      <c r="R143" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -9042,10 +9042,10 @@
         </is>
       </c>
       <c r="Q144" t="n">
+        <v>0</v>
+      </c>
+      <c r="R144" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R144" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -9099,10 +9099,10 @@
         </is>
       </c>
       <c r="Q145" t="n">
+        <v>0</v>
+      </c>
+      <c r="R145" t="n">
         <v>200000</v>
-      </c>
-      <c r="R145" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -9156,10 +9156,10 @@
         </is>
       </c>
       <c r="Q146" t="n">
+        <v>0</v>
+      </c>
+      <c r="R146" t="n">
         <v>30980000</v>
-      </c>
-      <c r="R146" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -9213,10 +9213,10 @@
         </is>
       </c>
       <c r="Q147" t="n">
+        <v>0</v>
+      </c>
+      <c r="R147" t="n">
         <v>25655000</v>
-      </c>
-      <c r="R147" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="148">
@@ -9270,10 +9270,10 @@
         </is>
       </c>
       <c r="Q148" t="n">
+        <v>0</v>
+      </c>
+      <c r="R148" t="n">
         <v>66560000</v>
-      </c>
-      <c r="R148" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="149">
@@ -9327,10 +9327,10 @@
         </is>
       </c>
       <c r="Q149" t="n">
+        <v>0</v>
+      </c>
+      <c r="R149" t="n">
         <v>25464500</v>
-      </c>
-      <c r="R149" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -9384,10 +9384,10 @@
         </is>
       </c>
       <c r="Q150" t="n">
+        <v>0</v>
+      </c>
+      <c r="R150" t="n">
         <v>1202905</v>
-      </c>
-      <c r="R150" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -9441,10 +9441,10 @@
         </is>
       </c>
       <c r="Q151" t="n">
+        <v>0</v>
+      </c>
+      <c r="R151" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R151" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -9498,10 +9498,10 @@
         </is>
       </c>
       <c r="Q152" t="n">
+        <v>0</v>
+      </c>
+      <c r="R152" t="n">
         <v>14920000</v>
-      </c>
-      <c r="R152" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -9555,10 +9555,10 @@
         </is>
       </c>
       <c r="Q153" t="n">
+        <v>0</v>
+      </c>
+      <c r="R153" t="n">
         <v>8798400</v>
-      </c>
-      <c r="R153" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="154">
@@ -9612,10 +9612,10 @@
         </is>
       </c>
       <c r="Q154" t="n">
+        <v>0</v>
+      </c>
+      <c r="R154" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R154" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="155">
@@ -9669,10 +9669,10 @@
         </is>
       </c>
       <c r="Q155" t="n">
+        <v>0</v>
+      </c>
+      <c r="R155" t="n">
         <v>1203643</v>
-      </c>
-      <c r="R155" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="156">
@@ -9726,10 +9726,10 @@
         </is>
       </c>
       <c r="Q156" t="n">
+        <v>0</v>
+      </c>
+      <c r="R156" t="n">
         <v>66620</v>
-      </c>
-      <c r="R156" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="157">
@@ -9783,10 +9783,10 @@
         </is>
       </c>
       <c r="Q157" t="n">
+        <v>0</v>
+      </c>
+      <c r="R157" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R157" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="158">
@@ -9840,10 +9840,10 @@
         </is>
       </c>
       <c r="Q158" t="n">
+        <v>0</v>
+      </c>
+      <c r="R158" t="n">
         <v>2940000</v>
-      </c>
-      <c r="R158" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="159">
@@ -9897,10 +9897,10 @@
         </is>
       </c>
       <c r="Q159" t="n">
+        <v>0</v>
+      </c>
+      <c r="R159" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R159" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="160">
@@ -9954,10 +9954,10 @@
         </is>
       </c>
       <c r="Q160" t="n">
+        <v>0</v>
+      </c>
+      <c r="R160" t="n">
         <v>542000</v>
-      </c>
-      <c r="R160" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -10011,10 +10011,10 @@
         </is>
       </c>
       <c r="Q161" t="n">
+        <v>0</v>
+      </c>
+      <c r="R161" t="n">
         <v>2163814</v>
-      </c>
-      <c r="R161" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="162">
@@ -10068,10 +10068,10 @@
         </is>
       </c>
       <c r="Q162" t="n">
+        <v>0</v>
+      </c>
+      <c r="R162" t="n">
         <v>11974837</v>
-      </c>
-      <c r="R162" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="163">
@@ -10125,10 +10125,10 @@
         </is>
       </c>
       <c r="Q163" t="n">
+        <v>0</v>
+      </c>
+      <c r="R163" t="n">
         <v>1382535</v>
-      </c>
-      <c r="R163" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="164">
@@ -10182,10 +10182,10 @@
         </is>
       </c>
       <c r="Q164" t="n">
+        <v>0</v>
+      </c>
+      <c r="R164" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R164" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="165">
@@ -10239,10 +10239,10 @@
         </is>
       </c>
       <c r="Q165" t="n">
+        <v>0</v>
+      </c>
+      <c r="R165" t="n">
         <v>35359853</v>
-      </c>
-      <c r="R165" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="166">
@@ -10296,10 +10296,10 @@
         </is>
       </c>
       <c r="Q166" t="n">
+        <v>0</v>
+      </c>
+      <c r="R166" t="n">
         <v>13982612</v>
-      </c>
-      <c r="R166" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="167">
@@ -10353,10 +10353,10 @@
         </is>
       </c>
       <c r="Q167" t="n">
+        <v>0</v>
+      </c>
+      <c r="R167" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R167" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -10410,10 +10410,10 @@
         </is>
       </c>
       <c r="Q168" t="n">
+        <v>0</v>
+      </c>
+      <c r="R168" t="n">
         <v>10459632</v>
-      </c>
-      <c r="R168" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="169">
@@ -10467,10 +10467,10 @@
         </is>
       </c>
       <c r="Q169" t="n">
+        <v>0</v>
+      </c>
+      <c r="R169" t="n">
         <v>17000000</v>
-      </c>
-      <c r="R169" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="170">
@@ -10524,10 +10524,10 @@
         </is>
       </c>
       <c r="Q170" t="n">
+        <v>0</v>
+      </c>
+      <c r="R170" t="n">
         <v>74941121</v>
-      </c>
-      <c r="R170" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="171">
@@ -10581,10 +10581,10 @@
         </is>
       </c>
       <c r="Q171" t="n">
+        <v>0</v>
+      </c>
+      <c r="R171" t="n">
         <v>38460000</v>
-      </c>
-      <c r="R171" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="172">
@@ -10638,10 +10638,10 @@
         </is>
       </c>
       <c r="Q172" t="n">
+        <v>0</v>
+      </c>
+      <c r="R172" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R172" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="173">
@@ -10695,10 +10695,10 @@
         </is>
       </c>
       <c r="Q173" t="n">
+        <v>0</v>
+      </c>
+      <c r="R173" t="n">
         <v>7000000</v>
-      </c>
-      <c r="R173" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="174">
@@ -10752,10 +10752,10 @@
         </is>
       </c>
       <c r="Q174" t="n">
+        <v>0</v>
+      </c>
+      <c r="R174" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R174" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -11265,10 +11265,10 @@
         </is>
       </c>
       <c r="Q183" t="n">
+        <v>0</v>
+      </c>
+      <c r="R183" t="n">
         <v>100000</v>
-      </c>
-      <c r="R183" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="184">
@@ -11322,10 +11322,10 @@
         </is>
       </c>
       <c r="Q184" t="n">
+        <v>0</v>
+      </c>
+      <c r="R184" t="n">
         <v>6121132</v>
-      </c>
-      <c r="R184" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="185">
@@ -11379,10 +11379,10 @@
         </is>
       </c>
       <c r="Q185" t="n">
+        <v>0</v>
+      </c>
+      <c r="R185" t="n">
         <v>3541728</v>
-      </c>
-      <c r="R185" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="186">
@@ -11436,10 +11436,10 @@
         </is>
       </c>
       <c r="Q186" t="n">
+        <v>0</v>
+      </c>
+      <c r="R186" t="n">
         <v>22254062</v>
-      </c>
-      <c r="R186" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="187">
@@ -11493,10 +11493,10 @@
         </is>
       </c>
       <c r="Q187" t="n">
+        <v>0</v>
+      </c>
+      <c r="R187" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R187" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="188">
@@ -11550,10 +11550,10 @@
         </is>
       </c>
       <c r="Q188" t="n">
+        <v>0</v>
+      </c>
+      <c r="R188" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R188" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="189">
@@ -11607,10 +11607,10 @@
         </is>
       </c>
       <c r="Q189" t="n">
+        <v>0</v>
+      </c>
+      <c r="R189" t="n">
         <v>431809</v>
-      </c>
-      <c r="R189" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="190">
@@ -11664,10 +11664,10 @@
         </is>
       </c>
       <c r="Q190" t="n">
+        <v>0</v>
+      </c>
+      <c r="R190" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R190" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="191">
@@ -11721,10 +11721,10 @@
         </is>
       </c>
       <c r="Q191" t="n">
+        <v>0</v>
+      </c>
+      <c r="R191" t="n">
         <v>14356790</v>
-      </c>
-      <c r="R191" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="192">
@@ -11778,10 +11778,10 @@
         </is>
       </c>
       <c r="Q192" t="n">
+        <v>0</v>
+      </c>
+      <c r="R192" t="n">
         <v>1000</v>
-      </c>
-      <c r="R192" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="193">
@@ -11835,10 +11835,10 @@
         </is>
       </c>
       <c r="Q193" t="n">
+        <v>0</v>
+      </c>
+      <c r="R193" t="n">
         <v>1000</v>
-      </c>
-      <c r="R193" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="194">
@@ -12291,10 +12291,10 @@
         </is>
       </c>
       <c r="Q201" t="n">
+        <v>0</v>
+      </c>
+      <c r="R201" t="n">
         <v>50000000</v>
-      </c>
-      <c r="R201" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="202">
@@ -12348,10 +12348,10 @@
         </is>
       </c>
       <c r="Q202" t="n">
+        <v>0</v>
+      </c>
+      <c r="R202" t="n">
         <v>8151612</v>
-      </c>
-      <c r="R202" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="203">
@@ -12405,10 +12405,10 @@
         </is>
       </c>
       <c r="Q203" t="n">
+        <v>0</v>
+      </c>
+      <c r="R203" t="n">
         <v>7488179</v>
-      </c>
-      <c r="R203" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="204">
@@ -12462,10 +12462,10 @@
         </is>
       </c>
       <c r="Q204" t="n">
+        <v>0</v>
+      </c>
+      <c r="R204" t="n">
         <v>9608804</v>
-      </c>
-      <c r="R204" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="205">
@@ -12519,10 +12519,10 @@
         </is>
       </c>
       <c r="Q205" t="n">
+        <v>0</v>
+      </c>
+      <c r="R205" t="n">
         <v>8168067</v>
-      </c>
-      <c r="R205" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="206">
@@ -12576,10 +12576,10 @@
         </is>
       </c>
       <c r="Q206" t="n">
+        <v>0</v>
+      </c>
+      <c r="R206" t="n">
         <v>571386707</v>
-      </c>
-      <c r="R206" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="207">
@@ -12633,10 +12633,10 @@
         </is>
       </c>
       <c r="Q207" t="n">
+        <v>0</v>
+      </c>
+      <c r="R207" t="n">
         <v>15000000</v>
-      </c>
-      <c r="R207" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="208">
@@ -12690,10 +12690,10 @@
         </is>
       </c>
       <c r="Q208" t="n">
+        <v>0</v>
+      </c>
+      <c r="R208" t="n">
         <v>1406178</v>
-      </c>
-      <c r="R208" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="209">
@@ -12747,10 +12747,10 @@
         </is>
       </c>
       <c r="Q209" t="n">
+        <v>0</v>
+      </c>
+      <c r="R209" t="n">
         <v>19448656</v>
-      </c>
-      <c r="R209" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="210">
@@ -12804,10 +12804,10 @@
         </is>
       </c>
       <c r="Q210" t="n">
+        <v>0</v>
+      </c>
+      <c r="R210" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R210" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="211">
@@ -12861,10 +12861,10 @@
         </is>
       </c>
       <c r="Q211" t="n">
+        <v>0</v>
+      </c>
+      <c r="R211" t="n">
         <v>30000000</v>
-      </c>
-      <c r="R211" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="212">
@@ -12918,10 +12918,10 @@
         </is>
       </c>
       <c r="Q212" t="n">
+        <v>0</v>
+      </c>
+      <c r="R212" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R212" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="213">
@@ -12975,10 +12975,10 @@
         </is>
       </c>
       <c r="Q213" t="n">
+        <v>0</v>
+      </c>
+      <c r="R213" t="n">
         <v>4000000</v>
-      </c>
-      <c r="R213" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -13032,10 +13032,10 @@
         </is>
       </c>
       <c r="Q214" t="n">
+        <v>0</v>
+      </c>
+      <c r="R214" t="n">
         <v>4000000</v>
-      </c>
-      <c r="R214" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="215">
@@ -13089,10 +13089,10 @@
         </is>
       </c>
       <c r="Q215" t="n">
+        <v>0</v>
+      </c>
+      <c r="R215" t="n">
         <v>1000000</v>
-      </c>
-      <c r="R215" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="216">
@@ -13442,10 +13442,10 @@
         </is>
       </c>
       <c r="Q221" t="n">
+        <v>0</v>
+      </c>
+      <c r="R221" t="n">
         <v>8311374</v>
-      </c>
-      <c r="R221" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="222">
@@ -13499,10 +13499,10 @@
         </is>
       </c>
       <c r="Q222" t="n">
+        <v>0</v>
+      </c>
+      <c r="R222" t="n">
         <v>477508</v>
-      </c>
-      <c r="R222" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="223">

</xml_diff>